<commit_message>
Erabilera kasu berri bat.
</commit_message>
<xml_diff>
--- a/GI/ERRONKA.xlsx
+++ b/GI/ERRONKA.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\390401F\eclipse-workspace\T5E2Prog\GI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\390401F\eclipse-workspace\T4E3Prog\GI\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="21">
   <si>
     <t>Erabilera-kasuaren izena:</t>
   </si>
@@ -60,15 +60,6 @@
   </si>
   <si>
     <t>EK-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. 
-2. 
-3. 
-4.
-5. 
-6. 
-7. </t>
   </si>
   <si>
     <t>1. 
@@ -81,6 +72,31 @@
   </si>
   <si>
     <t>EK-03</t>
+  </si>
+  <si>
+    <t>Hasi saioa</t>
+  </si>
+  <si>
+    <t>Erabiltzailea sisteman identifikatzen da bere funtzioetara sartzeko.</t>
+  </si>
+  <si>
+    <t>Erabiltzailea (eta hedaduraz: Presi, Epaile, Administratzailea).</t>
+  </si>
+  <si>
+    <t>Erabiltzaileak aldez aurretik erregistratuta egon behar du datu-basean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Erabiltzaileak programa irekitzen du
+2. Erabiltzaileak bere erabiltzaile-izena eta pasahitza sartzen ditu.
+3. Sistemak kredentzialak baliozkotzen ditu.
+4. Sistemak Log-en erregistratzen du sarbidea (Include: Log fitxategian idatzi).
+5. Sistemak panel nagusira birbideratzen du, rolaren arabera. </t>
+  </si>
+  <si>
+    <t>Erabiltzaileak bere rolaren funtzio berezietarako sarbidea du.</t>
+  </si>
+  <si>
+    <t>Kredentzial okerrak: Datuak bat ez badatoz, sistemak errore-mezu bat erakusten du eta berriro saiatzeko aukera ematen du.</t>
   </si>
 </sst>
 </file>
@@ -166,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
@@ -184,6 +200,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -486,7 +505,9 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="C2" s="3"/>
       <c r="E2" s="3"/>
     </row>
@@ -509,7 +530,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
@@ -524,7 +545,9 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
+      <c r="A6" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="C6" s="5"/>
       <c r="E6" s="5"/>
     </row>
@@ -540,7 +563,9 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
+      <c r="A8" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="C8" s="5"/>
       <c r="E8" s="5"/>
     </row>
@@ -556,7 +581,9 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
+      <c r="A10" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="C10" s="5"/>
       <c r="E10" s="5"/>
     </row>
@@ -573,13 +600,13 @@
     </row>
     <row r="12" spans="1:5" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
@@ -594,7 +621,9 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
+      <c r="A14" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="C14" s="5"/>
       <c r="E14" s="5"/>
     </row>
@@ -610,7 +639,9 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="6"/>
+      <c r="A16" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="C16" s="6"/>
       <c r="E16" s="6"/>
     </row>

</xml_diff>

<commit_message>
Klase diagrama ondo ipini eta Erabilerakasuen dokumentazioa amaitu.
</commit_message>
<xml_diff>
--- a/GI/ERRONKA.xlsx
+++ b/GI/ERRONKA.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="44">
   <si>
     <t>Erabilera-kasuaren izena:</t>
   </si>
@@ -62,21 +62,9 @@
     <t>EK-02</t>
   </si>
   <si>
-    <t>1. 
-2. 
-3. 
-4.
-5. 
-6. 
-7.</t>
-  </si>
-  <si>
     <t>EK-03</t>
   </si>
   <si>
-    <t>Hasi saioa</t>
-  </si>
-  <si>
     <t>Erabiltzailea sisteman identifikatzen da bere funtzioetara sartzeko.</t>
   </si>
   <si>
@@ -84,26 +72,113 @@
   </si>
   <si>
     <t>Erabiltzaileak aldez aurretik erregistratuta egon behar du datu-basean.</t>
+  </si>
+  <si>
+    <t>Erabiltzaileak bere rolaren funtzio berezietarako sarbidea du.</t>
+  </si>
+  <si>
+    <t>Kredentzial okerrak: Datuak bat ez badatoz, sistemak errore-mezu bat erakusten du eta berriro saiatzeko aukera ematen du.</t>
+  </si>
+  <si>
+    <t>Presidenteak denboraldi berri bat prestazen eta martxan jartzen du.</t>
+  </si>
+  <si>
+    <t>Presi.</t>
+  </si>
+  <si>
+    <t>Presidenteak behar bezala hasi behar du saioa, eta aurreko denboraldia osatuta egon behar da.</t>
+  </si>
+  <si>
+    <t>1. Lehendakariak denboraldi berria sortzeko aukera hautatzen du.
+2. Sistemak denboraldi berri horretan parte hartuko duten taldeak eskatzen ditu.
+3. Lehendakariak sorrera baieztatzen du.
+4. Sistemak ekintza erregistratzen du (Include: Log fitxategian idatzi).</t>
+  </si>
+  <si>
+    <t>Denboraldia sortu da eta emaitzak gehitzeko prest dago.</t>
+  </si>
+  <si>
+    <t>Denboraldia sortzeko 6 talde aukeratzen ez badituzu, sistemak errore-mezu bat erakutsiko dizu, eta hura egiteko aukera emango dizu.</t>
+  </si>
+  <si>
+    <t>EK-04</t>
+  </si>
+  <si>
+    <t>Epaileak jokatutako partiden emaitzak erregistratzen ditu.</t>
+  </si>
+  <si>
+    <t>Epaile.</t>
+  </si>
+  <si>
+    <t>Epaileak behar bezala hasi behar du saioa, eta denboraldi bat hasita egon behar da jokatu gabeko partidekin.</t>
+  </si>
+  <si>
+    <t>Emaitza gorde egiten da eta sailkapena eguneratu egiten da.</t>
+  </si>
+  <si>
+    <t>Admin.</t>
+  </si>
+  <si>
+    <t>Hasi saioa.</t>
+  </si>
+  <si>
+    <t>Denboraldi berri bat hasieratu.</t>
+  </si>
+  <si>
+    <t>Emaitzak sartu.</t>
+  </si>
+  <si>
+    <t>Jokalari bat taldez aldatu</t>
+  </si>
+  <si>
+    <t>Administratzaileak jokalari batek taldez aldatzen du.</t>
+  </si>
+  <si>
+    <t>Administratzaileak behar bezala hasi behar du saioa, eta denboraldia hasi gabe egon behar da.</t>
+  </si>
+  <si>
+    <t>1. Epaileak emaitza berri bat sartzeko aukera hautatzen du.
+2. Dagokion partida hautatzen du.
+3. Partidaren emaitza sartzen du.
+4. Sistemak datuak koherenteak izatea baliozkotzen du.
+5. Sistemak ekintza erregistratzen du (Include: Log fitxategian idatzi).</t>
   </si>
   <si>
     <t xml:space="preserve">1. Erabiltzaileak programa irekitzen du
 2. Erabiltzaileak bere erabiltzaile-izena eta pasahitza sartzen ditu.
 3. Sistemak kredentzialak baliozkotzen ditu.
-4. Sistemak Log-en erregistratzen du sarbidea (Include: Log fitxategian idatzi).
+4. Sistemak sarbidea erregistratzen du (Include: Log fitxategian idatzi).
 5. Sistemak panel nagusira birbideratzen du, rolaren arabera. </t>
   </si>
   <si>
-    <t>Erabiltzaileak bere rolaren funtzio berezietarako sarbidea du.</t>
-  </si>
-  <si>
-    <t>Kredentzial okerrak: Datuak bat ez badatoz, sistemak errore-mezu bat erakusten du eta berriro saiatzeko aukera ematen du.</t>
+    <t>1. Administratzaileak jokalari batek taldez aldatzeko aukera hautatzen du.
+2. Taldez aldatuko den jokalariaren taldea hautatzen du.
+3. Taldez aldatuko den jokalaria hautatzen du.
+4. Jokalariaren talde berria hautatzen du.
+5. Sistemak datuak koherenteak izatea baliozkotzen du.
+6. Sistemak ekintza erregistratzen du (Include: Log fitxategian idatzi).</t>
+  </si>
+  <si>
+    <t>Aldaketa gorde egiten da eta taldeen zerrendak eguneratu egiten dira.</t>
+  </si>
+  <si>
+    <t>Datu baliogabeak: Ezinezko balioak sartuz gero (adibidez: zenbaki negatiboak), sistemak errore-mezu bat erakutsiko dizu, eta hura egiteko aukera emango dizu.</t>
+  </si>
+  <si>
+    <t>Taldez aldatzen den jokalaria berriro talde berbera sartzen saiatuz gero, sistemak errore-mezu bat erakutsiko dizu, eta hura egiteko aukera emango dizu.</t>
+  </si>
+  <si>
+    <t>Taldez aldatzen den jokalariaren talde berria jokalari gehiegi baditu, sistemak errore-mezu bat erakutsiko dizu, eta hura egiteko aukera emango dizu.</t>
+  </si>
+  <si>
+    <t>Taldez aldatzen den jokalariaren talde zaharra jokalari gutxiekin geratzen bada, sistemak errore-mezu bat erakutsiko dizu, eta hura egiteko aukera emango dizu.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,14 +201,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -184,26 +251,26 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -485,201 +552,346 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="85.109375" customWidth="1"/>
     <col min="3" max="3" width="85.109375" customWidth="1"/>
     <col min="5" max="5" width="85.109375" customWidth="1"/>
+    <col min="7" max="7" width="85.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" s="3"/>
+      <c r="E1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="F1" s="3"/>
+      <c r="G1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="B8" s="3"/>
+      <c r="C8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="B10" s="3"/>
+      <c r="C10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="3"/>
+      <c r="G12" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="B14" s="3"/>
+      <c r="C14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="3"/>
+      <c r="G14" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="E16" s="6"/>
-    </row>
-    <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="B16" s="3"/>
+      <c r="C16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="B17" s="3"/>
+      <c r="C17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="D17" s="3"/>
+      <c r="E17" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="C18" s="6"/>
-      <c r="E18" s="6"/>
-    </row>
-    <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="F17" s="3"/>
+      <c r="G17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="B19" s="3"/>
+      <c r="C19" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="D19" s="3"/>
+      <c r="E19" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="E20" s="2"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange algorithmName="SHA-512" hashValue="H3t9EXZDFh+vZlCZHHkUXWOICtBSx4TVIaJtWvf8q1xZr7HubdAWp/x9d92w4ZvqAkAc0Kk2WJdMwa0jfZN7JQ==" saltValue="nbSPWguz0U+MgedRXp8GWA==" spinCount="100000" sqref="A2 A4 A6 A8 A10 A12 A14 A16 A18 A20 C2 C4 C6 C8 C10 C12 C14 C16 C18 C20 E2 E4 E6 E8 E10 E12 E14 E16 E18 E20" name="ErabileraKasuDok"/>
+    <protectedRange algorithmName="SHA-512" hashValue="H3t9EXZDFh+vZlCZHHkUXWOICtBSx4TVIaJtWvf8q1xZr7HubdAWp/x9d92w4ZvqAkAc0Kk2WJdMwa0jfZN7JQ==" saltValue="nbSPWguz0U+MgedRXp8GWA==" spinCount="100000" sqref="A2 A4 A6 A8 A10 A12 A14 A16 A18 A20 C2 C4 C6 C8 C10 C12 C14 C16 C18 C20 E2 E4 E6 E8 E10 E12 E14 E16 E18 E20 G2 G4 G6 G8 G10 G12 G14 G16 G18 G20" name="ErabileraKasuDok"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>